<commit_message>
Actualización manual ERP manual - Informe Stock Sanitarios.xlsx - 22/08/2026 09:52:58
</commit_message>
<xml_diff>
--- a/Data_ERP/Informe Stock Sanitarios.xlsx
+++ b/Data_ERP/Informe Stock Sanitarios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\Sistema_Logistico_Peirano\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E17BCA74-62A2-455C-B84E-8479E906D8C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2B9782A4-7354-453C-8244-B24A918C46C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{5888EA3A-7165-4FE6-AE0A-B397685057B6}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{559AA498-00A5-4B6E-AF33-1B56925F4D98}"/>
   </bookViews>
   <sheets>
     <sheet name="200" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="47">
   <si>
     <t>cod_art</t>
   </si>
@@ -49,6 +49,12 @@
     <t>stk_nivel</t>
   </si>
   <si>
+    <t>est_1</t>
+  </si>
+  <si>
+    <t>est_8</t>
+  </si>
+  <si>
     <t>cod_unidad</t>
   </si>
   <si>
@@ -109,10 +115,10 @@
     <t>CERAMICA</t>
   </si>
   <si>
-    <t>BID103-1</t>
-  </si>
-  <si>
-    <t>BIDE 1 AGUJERO BLANCO LINEA URBAN</t>
+    <t>BID103-3</t>
+  </si>
+  <si>
+    <t>BIDE 3 AGUJEROS BLANCO LINEA URBAN</t>
   </si>
   <si>
     <t>00100</t>
@@ -127,12 +133,6 @@
     <t>SANITARIOS</t>
   </si>
   <si>
-    <t>BID103-3</t>
-  </si>
-  <si>
-    <t>BIDE 3 AGUJEROS BLANCO LINEA URBAN</t>
-  </si>
-  <si>
     <t>BID104-3</t>
   </si>
   <si>
@@ -143,6 +143,12 @@
   </si>
   <si>
     <t>LINEA STONE</t>
+  </si>
+  <si>
+    <t>CMP01</t>
+  </si>
+  <si>
+    <t>CAMPANA SLIM 60 CM 3 VELOCIDADES</t>
   </si>
   <si>
     <t>INO103-1</t>
@@ -590,11 +596,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1A40D54-5924-4739-8A6C-757DE956B577}">
-  <dimension ref="A1:T7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB51B76B-8A06-4B1F-8E4B-3C64058E2C41}">
+  <dimension ref="A1:V7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -655,13 +661,19 @@
       <c r="T1" t="s">
         <v>19</v>
       </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C2">
         <v>300</v>
@@ -679,28 +691,28 @@
         <v>300</v>
       </c>
       <c r="H2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
-      <c r="J2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>300</v>
+      </c>
+      <c r="L2" t="s">
+        <v>25</v>
       </c>
       <c r="M2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N2" t="s">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
       </c>
       <c r="O2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="P2" t="s">
         <v>27</v>
@@ -708,22 +720,28 @@
       <c r="Q2" t="s">
         <v>28</v>
       </c>
-      <c r="R2">
-        <v>0</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
+      <c r="R2" t="s">
+        <v>29</v>
+      </c>
+      <c r="S2" t="s">
+        <v>30</v>
       </c>
       <c r="T2">
         <v>0</v>
       </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C3">
         <v>200</v>
@@ -741,28 +759,28 @@
         <v>200</v>
       </c>
       <c r="H3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
-      <c r="J3" t="s">
-        <v>23</v>
-      </c>
-      <c r="K3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L3">
-        <v>0</v>
+      <c r="J3">
+        <v>200</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3" t="s">
+        <v>25</v>
       </c>
       <c r="M3" t="s">
-        <v>22</v>
-      </c>
-      <c r="N3" t="s">
-        <v>31</v>
+        <v>26</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="P3" t="s">
         <v>33</v>
@@ -770,87 +788,99 @@
       <c r="Q3" t="s">
         <v>34</v>
       </c>
-      <c r="R3">
-        <v>0</v>
-      </c>
-      <c r="S3">
-        <v>0</v>
+      <c r="R3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S3" t="s">
+        <v>36</v>
       </c>
       <c r="T3">
         <v>0</v>
       </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4">
+        <v>300</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>300</v>
+      </c>
+      <c r="H4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>164</v>
+      </c>
+      <c r="K4">
+        <v>136</v>
+      </c>
+      <c r="L4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M4" t="s">
+        <v>26</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P4" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>40</v>
+      </c>
+      <c r="R4" t="s">
         <v>35</v>
       </c>
-      <c r="B4" t="s">
+      <c r="S4" t="s">
         <v>36</v>
       </c>
-      <c r="C4">
-        <v>200</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>200</v>
-      </c>
-      <c r="H4" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4" t="s">
-        <v>22</v>
-      </c>
-      <c r="N4" t="s">
-        <v>31</v>
-      </c>
-      <c r="O4" t="s">
-        <v>32</v>
-      </c>
-      <c r="P4" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>34</v>
-      </c>
-      <c r="R4">
-        <v>0</v>
-      </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
       <c r="T4">
         <v>0</v>
       </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C5">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -862,54 +892,60 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="H5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I5">
         <v>0</v>
       </c>
-      <c r="J5" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" t="s">
-        <v>24</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
+      <c r="J5">
+        <v>80</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="s">
+        <v>25</v>
       </c>
       <c r="M5" t="s">
-        <v>22</v>
-      </c>
-      <c r="N5" t="s">
-        <v>39</v>
+        <v>26</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="P5" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="Q5" t="s">
-        <v>34</v>
-      </c>
-      <c r="R5">
-        <v>0</v>
-      </c>
-      <c r="S5">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="R5" t="s">
+        <v>24</v>
+      </c>
+      <c r="S5" t="s">
+        <v>24</v>
       </c>
       <c r="T5">
         <v>0</v>
       </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C6">
         <v>440</v>
@@ -927,28 +963,28 @@
         <v>440</v>
       </c>
       <c r="H6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
-      <c r="J6" t="s">
-        <v>23</v>
-      </c>
-      <c r="K6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
+      <c r="J6">
+        <v>440</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6" t="s">
+        <v>25</v>
       </c>
       <c r="M6" t="s">
-        <v>22</v>
-      </c>
-      <c r="N6" t="s">
-        <v>31</v>
+        <v>26</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
       </c>
       <c r="O6" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="P6" t="s">
         <v>33</v>
@@ -956,22 +992,28 @@
       <c r="Q6" t="s">
         <v>34</v>
       </c>
-      <c r="R6">
-        <v>0</v>
-      </c>
-      <c r="S6">
-        <v>0</v>
+      <c r="R6" t="s">
+        <v>35</v>
+      </c>
+      <c r="S6" t="s">
+        <v>36</v>
       </c>
       <c r="T6">
         <v>0</v>
       </c>
+      <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C7">
         <v>440</v>
@@ -989,28 +1031,28 @@
         <v>440</v>
       </c>
       <c r="H7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
-      <c r="J7" t="s">
-        <v>23</v>
-      </c>
-      <c r="K7" t="s">
-        <v>24</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
+      <c r="J7">
+        <v>440</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7" t="s">
+        <v>25</v>
       </c>
       <c r="M7" t="s">
-        <v>22</v>
-      </c>
-      <c r="N7" t="s">
-        <v>31</v>
+        <v>26</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="P7" t="s">
         <v>33</v>
@@ -1018,13 +1060,19 @@
       <c r="Q7" t="s">
         <v>34</v>
       </c>
-      <c r="R7">
-        <v>0</v>
-      </c>
-      <c r="S7">
-        <v>0</v>
+      <c r="R7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S7" t="s">
+        <v>36</v>
       </c>
       <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="U7">
+        <v>0</v>
+      </c>
+      <c r="V7">
         <v>0</v>
       </c>
     </row>

</xml_diff>